<commit_message>
updating data gen pipeline
</commit_message>
<xml_diff>
--- a/data_generation/andes_cases/ieee39_full_ibrs.xlsx
+++ b/data_generation/andes_cases/ieee39_full_ibrs.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10118"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10208"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cloud9/Desktop/ETH Project/Working folder/03_Code/vis-ml/data_generation/andes_cases/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F203FC6-25B8-6B44-856F-460CE21A41C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{507A1034-FAEC-3243-84D7-0BF09B10759A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17180" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="15000" windowHeight="18900" firstSheet="6" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Bus" sheetId="1" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="523" uniqueCount="269">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="527" uniqueCount="269">
   <si>
     <t>idx</t>
   </si>
@@ -3409,7 +3409,7 @@
         <v>205</v>
       </c>
       <c r="C2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D2" t="s">
         <v>205</v>
@@ -3471,7 +3471,7 @@
         <v>206</v>
       </c>
       <c r="C3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D3" t="s">
         <v>206</v>
@@ -3533,7 +3533,7 @@
         <v>207</v>
       </c>
       <c r="C4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D4" t="s">
         <v>207</v>
@@ -3595,7 +3595,7 @@
         <v>208</v>
       </c>
       <c r="C5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D5" t="s">
         <v>208</v>
@@ -3657,7 +3657,7 @@
         <v>209</v>
       </c>
       <c r="C6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D6" t="s">
         <v>209</v>
@@ -3719,7 +3719,7 @@
         <v>210</v>
       </c>
       <c r="C7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D7" t="s">
         <v>210</v>
@@ -3868,7 +3868,7 @@
         <v>228</v>
       </c>
       <c r="C2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D2" t="s">
         <v>228</v>
@@ -3942,7 +3942,7 @@
         <v>229</v>
       </c>
       <c r="C3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D3" t="s">
         <v>229</v>
@@ -4016,7 +4016,7 @@
         <v>230</v>
       </c>
       <c r="C4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D4" t="s">
         <v>230</v>
@@ -4090,7 +4090,7 @@
         <v>231</v>
       </c>
       <c r="C5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D5" t="s">
         <v>231</v>
@@ -4164,7 +4164,7 @@
         <v>232</v>
       </c>
       <c r="C6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D6" t="s">
         <v>232</v>
@@ -4238,7 +4238,7 @@
         <v>233</v>
       </c>
       <c r="C7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D7" t="s">
         <v>233</v>
@@ -4772,7 +4772,7 @@
         <v>0.8</v>
       </c>
       <c r="K2">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.2">
@@ -4842,7 +4842,7 @@
         <v>0.8</v>
       </c>
       <c r="K4">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.2">
@@ -4877,7 +4877,7 @@
         <v>0.8</v>
       </c>
       <c r="K5">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.2">
@@ -4912,7 +4912,7 @@
         <v>0.8</v>
       </c>
       <c r="K6">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.2">
@@ -4947,7 +4947,7 @@
         <v>0.8</v>
       </c>
       <c r="K7">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.2">
@@ -4982,7 +4982,7 @@
         <v>0.8</v>
       </c>
       <c r="K8">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.2">
@@ -5017,7 +5017,7 @@
         <v>0.8</v>
       </c>
       <c r="K9">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.2">
@@ -5087,7 +5087,7 @@
         <v>0.8</v>
       </c>
       <c r="K11">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.2">
@@ -5122,7 +5122,7 @@
         <v>0.8</v>
       </c>
       <c r="K12">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.2">
@@ -5157,7 +5157,7 @@
         <v>0.8</v>
       </c>
       <c r="K13">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.2">
@@ -5192,7 +5192,7 @@
         <v>0.8</v>
       </c>
       <c r="K14">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.2">
@@ -5227,7 +5227,7 @@
         <v>0.8</v>
       </c>
       <c r="K15">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.2">
@@ -5262,7 +5262,7 @@
         <v>0.8</v>
       </c>
       <c r="K16">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.2">
@@ -5297,7 +5297,7 @@
         <v>0.8</v>
       </c>
       <c r="K17">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.2">
@@ -5332,7 +5332,7 @@
         <v>0.8</v>
       </c>
       <c r="K18">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.2">
@@ -5367,7 +5367,7 @@
         <v>0.8</v>
       </c>
       <c r="K19">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.2">
@@ -10182,6 +10182,9 @@
       <c r="F2">
         <v>1</v>
       </c>
+      <c r="G2" t="s">
+        <v>268</v>
+      </c>
       <c r="H2">
         <v>1040</v>
       </c>
@@ -10189,10 +10192,10 @@
         <v>50</v>
       </c>
       <c r="J2">
-        <v>0.01</v>
+        <v>0.05</v>
       </c>
       <c r="K2">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="L2">
         <v>0</v>
@@ -10259,6 +10262,9 @@
       <c r="F3">
         <v>6</v>
       </c>
+      <c r="G3" t="s">
+        <v>268</v>
+      </c>
       <c r="H3">
         <v>1085.7</v>
       </c>
@@ -10266,10 +10272,10 @@
         <v>50</v>
       </c>
       <c r="J3">
-        <v>0.01</v>
+        <v>0.05</v>
       </c>
       <c r="K3">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="L3">
         <v>0</v>
@@ -10336,6 +10342,9 @@
       <c r="F4">
         <v>8</v>
       </c>
+      <c r="G4" t="s">
+        <v>268</v>
+      </c>
       <c r="H4">
         <v>970.2</v>
       </c>
@@ -10343,10 +10352,10 @@
         <v>50</v>
       </c>
       <c r="J4">
-        <v>0.01</v>
+        <v>0.05</v>
       </c>
       <c r="K4">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="L4">
         <v>0</v>
@@ -10413,6 +10422,9 @@
       <c r="F5">
         <v>9</v>
       </c>
+      <c r="G5" t="s">
+        <v>268</v>
+      </c>
       <c r="H5">
         <v>1684.1</v>
       </c>
@@ -10420,10 +10432,10 @@
         <v>50</v>
       </c>
       <c r="J5">
-        <v>0.01</v>
+        <v>0.05</v>
       </c>
       <c r="K5">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="L5">
         <v>0</v>
@@ -10472,6 +10484,7 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>